<commit_message>
Mimari & Altyapı: config.py ile merkezi parametre yönetimi ve logging_setup.py ile güvenli hata yönetimi eklendi. Performans: ProcessPoolExecutor kullanılarak çoklu çekirdek (multiprocessing) ile batch işleme hızı artırıldı. - Morfolojik & Kalite Kontrol: Hücre ortalama alan hesaplaması, kenar hücre (border cell) eleme filtresi ve Laplacian varyans tabanlı bulanıklık tespiti (QC) entegre edildi. - Arayüz (UI): Streamlit tabanlı interaktif dashboard oluşturuldu. Canlı parametre ayarı (Dev Mode), Plotly ile veri görselleştirme ve rapor indirme özellikleri eklendi. - AI Veri Hattı: Tespit edilen WBC hücrelerinin otomatik olarak kırpılması, galeride sergilenmesi ve ML modelleri için ZIP formatında dışa aktarılması (Patch Extraction) sağlandı.
</commit_message>
<xml_diff>
--- a/output/kan_sayim_raporu.xlsx
+++ b/output/kan_sayim_raporu.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,6 +450,21 @@
           <t>Toplam Hücre Sayısı</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Ortalama WBC Alanı (px)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Ortalama RBC Alanı (px)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Netlik Skoru</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -458,13 +473,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C2" t="n">
-        <v>259</v>
+        <v>244</v>
       </c>
       <c r="D2" t="n">
-        <v>273</v>
+        <v>256</v>
+      </c>
+      <c r="E2" t="n">
+        <v>4631.38</v>
+      </c>
+      <c r="F2" t="n">
+        <v>110.68</v>
+      </c>
+      <c r="G2" t="n">
+        <v>8.92</v>
       </c>
     </row>
   </sheetData>
@@ -510,13 +534,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C2" t="n">
-        <v>259</v>
+        <v>244</v>
       </c>
       <c r="D2" t="n">
-        <v>273</v>
+        <v>256</v>
       </c>
     </row>
     <row r="3">
@@ -526,13 +550,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C3" t="n">
-        <v>259</v>
+        <v>244</v>
       </c>
       <c r="D3" t="n">
-        <v>273</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4">
@@ -542,13 +566,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C4" t="n">
-        <v>259</v>
+        <v>244</v>
       </c>
       <c r="D4" t="n">
-        <v>273</v>
+        <v>256</v>
       </c>
     </row>
   </sheetData>

</xml_diff>